<commit_message>
Actualiza dos indicadores con registros
</commit_message>
<xml_diff>
--- a/Data/LISTADO DE INDICADORES A ACTUALIZAR.xlsx
+++ b/Data/LISTADO DE INDICADORES A ACTUALIZAR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shari\Dropbox\UMAD\Sociodemografico\GITHUB DEFINITIVOS\Piso-I-Demografia\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D39A46F-E8FE-47E7-9372-A4EEE05FC2A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C955B5A6-A22C-47DC-8F14-E5DDC0B2A391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="150" yWindow="160" windowWidth="19120" windowHeight="10080" xr2:uid="{4A99605D-6FD6-4335-B9D1-ADD9FB504937}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{4A99605D-6FD6-4335-B9D1-ADD9FB504937}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="89">
   <si>
     <t>nombre indicador</t>
   </si>
@@ -101,9 +101,6 @@
     <t>MSP</t>
   </si>
   <si>
-    <t>SI</t>
-  </si>
-  <si>
     <t>Tasa Global de Fecundidad</t>
   </si>
   <si>
@@ -185,9 +182,6 @@
     <t>Tasa de fecundidad adolescente observada  (por mil) por departamento (1996-2021)</t>
   </si>
   <si>
-    <t>MSP  y INE -Estimaciones y proyecciones de población. Revisión, 2013</t>
-  </si>
-  <si>
     <t>Tasa de mortalidad neonatal (por 1.000 nacidos vivos) 1984-2021</t>
   </si>
   <si>
@@ -299,13 +293,16 @@
     <t>Si</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>1996-2023</t>
   </si>
   <si>
     <t>1984-2023</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si </t>
   </si>
 </sst>
 </file>
@@ -723,13 +720,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0414EEED-C8C4-4D5C-B970-C53579FD16CC}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:H175"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="75.54296875" style="7" customWidth="1"/>
     <col min="2" max="2" width="12" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13.90625" style="7" customWidth="1"/>
+    <col min="3" max="3" width="59" style="7" bestFit="1" customWidth="1"/>
     <col min="4" max="7" width="9.08984375" style="7" customWidth="1"/>
     <col min="255" max="256" width="9.08984375" customWidth="1"/>
     <col min="257" max="257" width="92.08984375" customWidth="1"/>
@@ -1065,7 +1061,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -1082,7 +1078,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>9</v>
       </c>
@@ -1099,7 +1095,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
@@ -1116,7 +1112,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
@@ -1133,7 +1129,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
@@ -1150,7 +1146,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>15</v>
       </c>
@@ -1167,7 +1163,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>16</v>
       </c>
@@ -1184,7 +1180,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>17</v>
       </c>
@@ -1201,7 +1197,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>18</v>
       </c>
@@ -1223,7 +1219,7 @@
         <v>19</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>20</v>
@@ -1232,49 +1228,49 @@
         <v>1</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="D12" s="4">
         <v>1</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D13" s="4">
         <v>1</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>7</v>
@@ -1283,15 +1279,15 @@
         <v>1</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>20</v>
@@ -1300,15 +1296,15 @@
         <v>1</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>28</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>7</v>
@@ -1320,9 +1316,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>11</v>
@@ -1337,9 +1333,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>11</v>
@@ -1354,9 +1350,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>11</v>
@@ -1371,12 +1367,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>7</v>
@@ -1388,12 +1384,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>7</v>
@@ -1405,9 +1401,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>6</v>
@@ -1422,9 +1418,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>6</v>
@@ -1439,9 +1435,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>6</v>
@@ -1456,9 +1452,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>6</v>
@@ -1473,9 +1469,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>6</v>
@@ -1490,9 +1486,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>6</v>
@@ -1507,9 +1503,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>6</v>
@@ -1524,9 +1520,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>6</v>
@@ -1541,9 +1537,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>6</v>
@@ -1558,9 +1554,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>6</v>
@@ -1575,9 +1571,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>6</v>
@@ -1592,9 +1588,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:8" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>6</v>
@@ -1609,9 +1605,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:8" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>6</v>
@@ -1626,9 +1622,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:8" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>6</v>
@@ -1645,92 +1641,92 @@
     </row>
     <row r="36" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="D36" s="4">
         <v>1</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="37" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="D37" s="6">
         <v>1</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="38" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="D38" s="6">
         <v>1</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="39" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="D39" s="6">
         <v>1</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="40" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D40" s="6">
         <v>1</v>
       </c>
-      <c r="E40" s="6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+      <c r="E40" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B41" s="2">
         <v>2011</v>
@@ -1745,9 +1741,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="1:8" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B42" s="2">
         <v>2011</v>
@@ -1762,9 +1758,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B43" s="2">
         <v>2011</v>
@@ -1780,9 +1776,9 @@
       </c>
       <c r="H43" s="8"/>
     </row>
-    <row r="44" spans="1:8" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B44" s="2">
         <v>2011</v>
@@ -1797,9 +1793,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="1:8" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A45" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B45" s="2">
         <v>2011</v>
@@ -1814,9 +1810,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="1:8" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A46" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B46" s="2">
         <v>2011</v>
@@ -1831,9 +1827,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:8" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A47" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B47" s="2"/>
       <c r="C47" s="9"/>
@@ -1844,9 +1840,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:8" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A48" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B48" s="2"/>
       <c r="C48" s="9"/>
@@ -1857,9 +1853,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="49" spans="1:5" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A49" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B49" s="2"/>
       <c r="C49" s="9"/>
@@ -1870,9 +1866,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:5" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A50" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B50" s="2"/>
       <c r="C50" s="9"/>
@@ -1883,9 +1879,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="1:5" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A51" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B51" s="2"/>
       <c r="C51" s="9"/>
@@ -1896,9 +1892,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="52" spans="1:5" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A52" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B52" s="2"/>
       <c r="C52" s="9"/>
@@ -1909,9 +1905,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="53" spans="1:5" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A53" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B53" s="2"/>
       <c r="C53" s="9"/>
@@ -1922,9 +1918,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="1:5" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A54" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B54" s="2"/>
       <c r="C54" s="9"/>
@@ -1935,9 +1931,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="55" spans="1:5" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A55" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B55" s="2"/>
       <c r="C55" s="9"/>
@@ -1950,37 +1946,37 @@
     </row>
     <row r="56" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A56" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B56" s="2"/>
       <c r="C56" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D56" s="6">
         <v>1</v>
       </c>
-      <c r="E56" s="6" t="s">
-        <v>21</v>
+      <c r="E56" s="4" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="57" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A57" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B57" s="2"/>
       <c r="C57" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D57" s="6">
         <v>1</v>
       </c>
-      <c r="E57" s="6" t="s">
-        <v>21</v>
+      <c r="E57" s="4" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="58" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A58" s="6" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B58" s="2"/>
       <c r="C58" s="9" t="s">
@@ -1989,13 +1985,13 @@
       <c r="D58" s="6">
         <v>1</v>
       </c>
-      <c r="E58" s="6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+      <c r="E58" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A59" s="6" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B59" s="2"/>
       <c r="C59" s="9" t="s">
@@ -2004,13 +2000,13 @@
       <c r="D59" s="6">
         <v>1</v>
       </c>
-      <c r="E59" s="6" t="s">
+      <c r="E59" s="4" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="60" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A60" s="6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B60" s="2"/>
       <c r="C60" s="9" t="s">
@@ -2019,13 +2015,13 @@
       <c r="D60" s="6">
         <v>1</v>
       </c>
-      <c r="E60" s="6" t="s">
-        <v>21</v>
+      <c r="E60" s="4" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C61" s="10" t="s">
         <v>20</v>
@@ -2033,27 +2029,27 @@
       <c r="D61" s="7">
         <v>1</v>
       </c>
-      <c r="E61" s="6" t="s">
-        <v>86</v>
+      <c r="E61" s="4" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D62" s="7">
         <v>1</v>
       </c>
-      <c r="E62" s="6" t="s">
-        <v>86</v>
+      <c r="E62" s="4" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C63" s="10" t="s">
         <v>20</v>
@@ -2061,13 +2057,13 @@
       <c r="D63" s="7">
         <v>1</v>
       </c>
-      <c r="E63" s="6" t="s">
-        <v>86</v>
+      <c r="E63" s="4" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C64" s="10" t="s">
         <v>20</v>
@@ -2075,64 +2071,64 @@
       <c r="D64" s="7">
         <v>1</v>
       </c>
-      <c r="E64" s="6" t="s">
-        <v>86</v>
+      <c r="E64" s="4" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="C65" s="10" t="s">
-        <v>23</v>
+        <v>77</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="D65" s="7">
         <v>1</v>
       </c>
-      <c r="E65" s="6" t="s">
-        <v>86</v>
+      <c r="E65" s="4" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C66" s="10" t="s">
-        <v>23</v>
+        <v>78</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="D66" s="7">
         <v>1</v>
       </c>
-      <c r="E66" s="6" t="s">
-        <v>86</v>
+      <c r="E66" s="4" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D67" s="7">
         <v>1</v>
       </c>
-      <c r="E67" s="6" t="s">
-        <v>86</v>
+      <c r="E67" s="4" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D68" s="7">
         <v>1</v>
       </c>
-      <c r="E68" s="6" t="s">
-        <v>86</v>
+      <c r="E68" s="4" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
@@ -2558,23 +2554,16 @@
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A175" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C175" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E68" xr:uid="{0414EEED-C8C4-4D5C-B970-C53579FD16CC}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="Si"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>